<commit_message>
Add presentation slides and references for fuel requirement estimation project
- Created a new LaTeX presentation (Final Slides.tex) detailing the pilot machine learning model for fuel requirement estimation in agricultural mechanization.
- Included sections on the problem, goals, data, methodology, results, and future work.
- Added a new BibTeX file (references.bib) containing relevant literature and resources for the project.
</commit_message>
<xml_diff>
--- a/Mini-Project/Agricultural Machinery Inventory from ABEMIS/Regression Parameters Output V3/LIME_Explanations.xlsx
+++ b/Mini-Project/Agricultural Machinery Inventory from ABEMIS/Regression Parameters Output V3/LIME_Explanations.xlsx
@@ -579,31 +579,31 @@
         <v>5.24</v>
       </c>
       <c r="E2" t="n">
-        <v>3.745857619047619</v>
+        <v>3.74585761904762</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.629341880476044</v>
+        <v>-2.630818815443216</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.4151278467526283</v>
+        <v>-0.420394993991814</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3251303683682722</v>
+        <v>0.3249725133878847</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.2697987129041038</v>
+        <v>-0.2688972837096559</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.2403597221107001</v>
+        <v>-0.2392986531231718</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.2144158118874803</v>
+        <v>-0.2278124071657639</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.2056609639604719</v>
+        <v>-0.2016660539763997</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.029615318852067</v>
+        <v>-0.02652684317571818</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
@@ -638,32 +638,32 @@
         <v>3.56</v>
       </c>
       <c r="E3" t="n">
-        <v>4.114252129629628</v>
+        <v>4.11425212962963</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.726557016477952</v>
+        <v>-2.728738055252629</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.04208867020285829</v>
+        <v>-0.04721123056588632</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3165455051371647</v>
+        <v>0.3167411855179946</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>0.148366254312576</v>
+        <v>0.1482706031401505</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.3835148978361831</v>
+        <v>-0.3963711889304313</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.1498019988650563</v>
+        <v>-0.1471790841041385</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.1966729936400423</v>
+        <v>-0.1943259555935131</v>
       </c>
       <c r="N3" t="n">
-        <v>0.04097845394592443</v>
+        <v>0.04063552895853018</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
@@ -704,31 +704,31 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>-0.1382628109618311</v>
+        <v>-0.1387087844015012</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.1851806129869198</v>
+        <v>-0.1981275602268284</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>-2.766833808720382</v>
+        <v>-2.768421769664014</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.9373423706886579</v>
+        <v>-0.9398536720443654</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3052812189641328</v>
+        <v>0.3091156042751244</v>
       </c>
       <c r="R4" t="n">
-        <v>0.1311526289870951</v>
+        <v>0.1350150464618997</v>
       </c>
       <c r="S4" t="n">
-        <v>0.01313075565779121</v>
+        <v>0.0119827252279117</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.001060544947477787</v>
+        <v>-0.0001500189625960924</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
@@ -760,29 +760,29 @@
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>-0.2178129035036614</v>
+        <v>-0.2227330902579061</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1029084738435933</v>
+        <v>0.1035502766240306</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>0.05494184725148955</v>
+        <v>0.05559154654830763</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.6403450696701748</v>
+        <v>-0.6531138098414819</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.4910469671904254</v>
+        <v>-0.4869146589043479</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.2188302229213667</v>
+        <v>-0.2165547705896562</v>
       </c>
       <c r="N5" t="n">
-        <v>-0.003660055932978632</v>
+        <v>-0.003921138128480573</v>
       </c>
       <c r="O5" t="n">
-        <v>-2.632118706107784</v>
+        <v>-2.634213416627437</v>
       </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
@@ -815,29 +815,29 @@
         <v>1.82</v>
       </c>
       <c r="E6" t="n">
-        <v>2.09599873015873</v>
+        <v>2.095998730158729</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>-0.2251748593526987</v>
+        <v>-0.2301911533196634</v>
       </c>
       <c r="H6" t="n">
-        <v>0.08107271896926936</v>
+        <v>0.07981500378866208</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.4828988562331128</v>
+        <v>-0.4822595504112216</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0352653716069657</v>
+        <v>-0.03516477531779141</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.5865594070236808</v>
+        <v>-0.5989331284369336</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.2198757623924245</v>
+        <v>-0.2162697664090322</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.09763213928933107</v>
+        <v>-0.09543732866481727</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
@@ -847,7 +847,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="n">
-        <v>-3.683823530265084</v>
+        <v>-3.686602174393012</v>
       </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
@@ -878,25 +878,25 @@
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>-0.3874603932119411</v>
+        <v>-0.3933377653867235</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07326770402710428</v>
+        <v>0.07343072783266087</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.3594522262454979</v>
+        <v>-0.3586070803444009</v>
       </c>
       <c r="J7" t="n">
-        <v>0.02218699050647747</v>
+        <v>0.02342826437668341</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.3330354260581576</v>
+        <v>-0.346619262222211</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.3235072922519838</v>
+        <v>-0.320456946022016</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.02749941920717533</v>
+        <v>-0.0243425277822412</v>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
@@ -906,7 +906,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="n">
-        <v>-3.822776330981053</v>
+        <v>-3.825907945667393</v>
       </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
@@ -933,7 +933,7 @@
         <v>6.43</v>
       </c>
       <c r="E8" t="n">
-        <v>8.810385328652826</v>
+        <v>8.810385328652824</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -944,33 +944,33 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>0.04955229263688482</v>
+        <v>0.04826153569381765</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>0.03234829081965868</v>
+        <v>0.03516486769974345</v>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
-        <v>-0.1904826283162094</v>
+        <v>-0.1913833709902212</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>9.141960471234805</v>
+        <v>9.147203808496091</v>
       </c>
       <c r="W8" t="n">
-        <v>-0.6043264951701934</v>
+        <v>-0.607176458761097</v>
       </c>
       <c r="X8" t="n">
-        <v>0.2552590922922839</v>
+        <v>0.2681999371973195</v>
       </c>
       <c r="Y8" t="n">
-        <v>-0.2022316893359316</v>
+        <v>-0.2022481792414225</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.1757186046026938</v>
+        <v>0.169586244495805</v>
       </c>
       <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
@@ -992,38 +992,38 @@
         <v>1.9</v>
       </c>
       <c r="E9" t="n">
-        <v>1.779066433381433</v>
+        <v>1.778319052429052</v>
       </c>
       <c r="F9" t="n">
-        <v>-2.627619567058812</v>
+        <v>-2.629547277344927</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>-0.04759631285374438</v>
+        <v>-0.04706314197080702</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.2912703607912473</v>
+        <v>-0.3032222620248808</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
-        <v>-0.7805855633712772</v>
+        <v>-0.780937815431144</v>
       </c>
       <c r="Q9" t="n">
-        <v>-0.1237650419987579</v>
+        <v>-0.1207796752586052</v>
       </c>
       <c r="R9" t="n">
-        <v>-0.2068790185453525</v>
+        <v>-0.2044946333665076</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.354594631360816</v>
+        <v>-0.3555533287193987</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.1552501271831163</v>
+        <v>-0.1547329926275443</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
         <v>8.25</v>
       </c>
       <c r="E10" t="n">
-        <v>8.194272632275137</v>
+        <v>8.183505965608468</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -1064,33 +1064,33 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
-        <v>-0.7479748182320073</v>
+        <v>-0.7487303292655223</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.1603056290139475</v>
+        <v>0.1640616531249567</v>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
-        <v>-0.2646001399074895</v>
+        <v>-0.2657427864752782</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>9.300306070768391</v>
+        <v>9.305525806399229</v>
       </c>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="n">
-        <v>0.359629771436013</v>
+        <v>0.3714603208659301</v>
       </c>
       <c r="Y10" t="n">
-        <v>-0.07797909450893037</v>
+        <v>-0.078353664258367</v>
       </c>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="n">
-        <v>0.9219315237491722</v>
+        <v>0.9206345506499337</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.3687809535338294</v>
+        <v>0.3729719224889272</v>
       </c>
       <c r="AC10" t="inlineStr"/>
     </row>
@@ -1124,33 +1124,33 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>0.1544844153225176</v>
+        <v>0.1579828703094102</v>
       </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
-        <v>-0.3037465098661606</v>
+        <v>-0.304297599320586</v>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>9.637356025895732</v>
+        <v>9.643630757640178</v>
       </c>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="n">
-        <v>0.2932439472403685</v>
+        <v>0.3066636769050058</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.09681110445802561</v>
+        <v>0.09729163432684355</v>
       </c>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="n">
-        <v>0.9312556858183</v>
+        <v>0.9283680159985847</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.4003957104844746</v>
+        <v>0.4051018570465884</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.777842879159116</v>
+        <v>1.778092981830971</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update agricultural machinery inventory project files and improve model performance
- Updated various PNG and Excel files in the Analytics Output and Regression Parameters directories to reflect the latest analysis results.
- Deleted outdated AMTEC extracted batch files to streamline the dataset.
- Revised the Final Paper and Final Slides documents to correct the number of cleaned training records from 378 to 376, reflecting the latest data processing outcomes.
- Enhanced model performance metrics in the paper, with Random Forest achieving R² = 0.916, MAE = 0.95 L/h, and RMSE = 1.53 L/h.
- Adjusted figures and captions in the documents to align with the updated dataset and results.
</commit_message>
<xml_diff>
--- a/Mini-Project/Agricultural Machinery Inventory from ABEMIS/Regression Parameters Output V3/LIME_Explanations.xlsx
+++ b/Mini-Project/Agricultural Machinery Inventory from ABEMIS/Regression Parameters Output V3/LIME_Explanations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC11"/>
+  <dimension ref="A1:AF11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,44 +444,44 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>lime_7.46 &lt; power_kw &lt;= 10.49</t>
+          <t>lime_7.45 &lt; power_kw &lt;= 10.43</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>lime_0.33 &lt; abemis_dominant_region_share &lt;= 0.97</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>lime_machinery_family_code=Stationary Engine / Irrigation</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>lime_0.33 &lt; abemis_dominant_region_share &lt;= 0.97</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>lime_analysis_subset_code=Dataset B - Stationary and Processing</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>lime_abemis_total_count &lt;= 4897.00</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>lime_machinery_type_code=Small Engine</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>lime_abemis_region_breadth &lt;= 16.00</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>lime_2012.00 &lt; year &lt;= 2013.00</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>lime_abemis_region_breadth &lt;= 16.00</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>lime_analysis_subset_code=Dataset B - Stationary and Processing</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>lime_abemis_total_count &lt;= 4897.00</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>lime_machinery_type_code=Small Engine</t>
-        </is>
-      </c>
       <c r="N1" t="inlineStr">
         <is>
           <t>lime_2013.00 &lt; year &lt;= 2014.00</t>
@@ -489,7 +489,7 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>lime_5.22 &lt; power_kw &lt;= 7.46</t>
+          <t>lime_5.22 &lt; power_kw &lt;= 7.45</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -509,63 +509,78 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>lime_machinery_type_code=Thresher</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>lime_abemis_dominant_region_share &lt;= 0.28</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>lime_machinery_type_code=Thresher</t>
-        </is>
-      </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>lime_abemis_total_count &gt; 18763.00</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>lime_0.28 &lt; abemis_dominant_region_share &lt;= 0.33</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>lime_machinery_type_code=Water Pump</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>lime_power_kw &lt;= 5.22</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>lime_power_kw &gt; 10.49</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>lime_power_kw &gt; 10.43</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>lime_machinery_type_code=Combine Harvester</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
         <is>
           <t>lime_machinery_family_code=Harvest Machinery</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>lime_analysis_subset_code=Dataset A - Field Machinery</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>lime_abemis_region_breadth &gt; 16.00</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>lime_machinery_type_code=Combine Harvester</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>lime_year &gt; 2014.00</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
         <is>
           <t>lime_machinery_type_code=Four-Wheel Tractor</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>lime_machinery_family_code=Mobile Field Machinery</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>lime_year &gt; 2014.00</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -579,31 +594,31 @@
         <v>5.24</v>
       </c>
       <c r="E2" t="n">
-        <v>3.74585761904762</v>
+        <v>4.773025097402599</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.630818815443216</v>
+        <v>-2.661632934002075</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.420394993991814</v>
+        <v>0.4047729002800384</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3249725133878847</v>
+        <v>-0.4016606959511843</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.2688972837096559</v>
+        <v>-0.3418159664713699</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.2392986531231718</v>
+        <v>-0.2689160773021237</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.2278124071657639</v>
+        <v>-0.2218776078799125</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.2016660539763997</v>
+        <v>-0.2070878373154598</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.02652684317571818</v>
+        <v>-0.1609686263057428</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
@@ -621,10 +636,13 @@
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -638,32 +656,32 @@
         <v>3.56</v>
       </c>
       <c r="E3" t="n">
-        <v>4.11425212962963</v>
+        <v>3.669926957671958</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.728738055252629</v>
+        <v>-2.773832901375084</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.04721123056588632</v>
+        <v>0.3896750403930276</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3167411855179946</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
+        <v>-0.0004381387909688706</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.4896020778838645</v>
+      </c>
       <c r="J3" t="n">
-        <v>0.1482706031401505</v>
+        <v>-0.2427537560580064</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.3963711889304313</v>
+        <v>-0.3306406434474226</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.1471790841041385</v>
-      </c>
-      <c r="M3" t="n">
-        <v>-0.1943259555935131</v>
-      </c>
+        <v>0.1897125632551027</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>0.04063552895853018</v>
+        <v>-0.07343393542540942</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
@@ -680,6 +698,9 @@
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -697,38 +718,38 @@
         <v>1.57</v>
       </c>
       <c r="E4" t="n">
-        <v>1.598838127705628</v>
+        <v>1.601455436137936</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="n">
-        <v>-0.1387087844015012</v>
-      </c>
-      <c r="K4" t="n">
-        <v>-0.1981275602268284</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>-0.3010538811758143</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>-0.1257995939520211</v>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>-2.768421769664014</v>
+        <v>-2.582607473340512</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.9398536720443654</v>
+        <v>-0.9384921060924487</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3091156042751244</v>
+        <v>0.3799108255880136</v>
       </c>
       <c r="R4" t="n">
-        <v>0.1350150464618997</v>
+        <v>0.09850368557041908</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0119827252279117</v>
+        <v>-0.05307788921290763</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.0001500189625960924</v>
+        <v>-0.02876307721986823</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
@@ -739,69 +760,75 @@
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Small Engine</t>
+          <t>Water Pump</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6.07</v>
+        <v>6.99</v>
       </c>
       <c r="D5" t="n">
-        <v>2.57</v>
+        <v>2.33</v>
       </c>
       <c r="E5" t="n">
-        <v>3.214718362840861</v>
+        <v>2.114847995245496</v>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>-0.2227330902579061</v>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>0.1035502766240306</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="n">
-        <v>0.05559154654830763</v>
-      </c>
-      <c r="K5" t="n">
-        <v>-0.6531138098414819</v>
-      </c>
+        <v>-0.1699799031126535</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.8378897691493004</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
-        <v>-0.4869146589043479</v>
-      </c>
-      <c r="M5" t="n">
-        <v>-0.2165547705896562</v>
-      </c>
+        <v>0.05579803239855275</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>-0.003921138128480573</v>
+        <v>-0.0193401822672192</v>
       </c>
       <c r="O5" t="n">
-        <v>-2.634213416627437</v>
+        <v>-2.558394613554744</v>
       </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>0.654387406805594</v>
+      </c>
+      <c r="V5" t="n">
+        <v>-0.5352146859463602</v>
+      </c>
+      <c r="W5" t="n">
+        <v>-0.2237185852481385</v>
+      </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -812,32 +839,32 @@
         <v>4.48</v>
       </c>
       <c r="D6" t="n">
-        <v>1.82</v>
+        <v>1.77</v>
       </c>
       <c r="E6" t="n">
-        <v>2.095998730158729</v>
+        <v>1.971947158489659</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>-0.2301911533196634</v>
+        <v>0.1761531222788708</v>
       </c>
       <c r="H6" t="n">
-        <v>0.07981500378866208</v>
+        <v>-0.172141519242678</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.4822595504112216</v>
+        <v>-0.6896876892120792</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.03516477531779141</v>
+        <v>-0.284476483704417</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.5989331284369336</v>
+        <v>-0.2640145784966079</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.2162697664090322</v>
+        <v>0.01322161741928922</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.09543732866481727</v>
+        <v>-0.3257296224171815</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
@@ -846,21 +873,24 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="n">
-        <v>-3.686602174393012</v>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
+      <c r="X6" t="n">
+        <v>-3.734259386708672</v>
+      </c>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -868,35 +898,35 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3.56</v>
+        <v>4.85</v>
       </c>
       <c r="D7" t="n">
-        <v>1.99</v>
+        <v>1.91</v>
       </c>
       <c r="E7" t="n">
-        <v>1.711668888888889</v>
+        <v>1.527651190476189</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>-0.3933377653867235</v>
+        <v>0.1594332923491214</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07343072783266087</v>
+        <v>-0.3648449619742762</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.3586070803444009</v>
+        <v>-0.444490632735192</v>
       </c>
       <c r="J7" t="n">
-        <v>0.02342826437668341</v>
+        <v>-0.3754166575747261</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.346619262222211</v>
+        <v>-0.1739852587978792</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.320456946022016</v>
+        <v>0.04110114625398473</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.0243425277822412</v>
+        <v>-0.2193374054738343</v>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
@@ -905,21 +935,24 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="n">
-        <v>-3.825907945667393</v>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
+      <c r="X7" t="n">
+        <v>-3.846095151394585</v>
+      </c>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -933,7 +966,7 @@
         <v>6.43</v>
       </c>
       <c r="E8" t="n">
-        <v>8.810385328652824</v>
+        <v>9.190078893791405</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -944,37 +977,40 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>0.04826153569381765</v>
+        <v>0.001625021065565524</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>0.03516486769974345</v>
+        <v>0.09477587786140802</v>
       </c>
       <c r="R8" t="inlineStr"/>
-      <c r="S8" t="n">
-        <v>-0.1913833709902212</v>
-      </c>
-      <c r="T8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="n">
+        <v>-0.239520687235515</v>
+      </c>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="n">
-        <v>9.147203808496091</v>
-      </c>
-      <c r="W8" t="n">
-        <v>-0.607176458761097</v>
-      </c>
-      <c r="X8" t="n">
-        <v>0.2681999371973195</v>
-      </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
       <c r="Y8" t="n">
-        <v>-0.2022481792414225</v>
+        <v>9.078615345035638</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.169586244495805</v>
-      </c>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
+        <v>0.5817687588766473</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>-0.5574726080823756</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.3579218512034312</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>-0.201855637347344</v>
+      </c>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -992,38 +1028,38 @@
         <v>1.9</v>
       </c>
       <c r="E9" t="n">
-        <v>1.778319052429052</v>
+        <v>1.71599557979058</v>
       </c>
       <c r="F9" t="n">
-        <v>-2.629547277344927</v>
+        <v>-2.678831593926442</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="n">
-        <v>-0.04706314197080702</v>
-      </c>
-      <c r="K9" t="n">
-        <v>-0.3032222620248808</v>
-      </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>-0.4384754074136887</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>-0.02089029825934417</v>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
-        <v>-0.780937815431144</v>
+        <v>-0.7622278598886364</v>
       </c>
       <c r="Q9" t="n">
-        <v>-0.1207796752586052</v>
+        <v>-0.05644710249183927</v>
       </c>
       <c r="R9" t="n">
-        <v>-0.2044946333665076</v>
+        <v>-0.1524470566218812</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.3555533287193987</v>
+        <v>-0.198652661973948</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.1547329926275443</v>
+        <v>-0.447080363708951</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
@@ -1034,6 +1070,9 @@
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1041,62 +1080,65 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Four-Wheel Tractor</t>
+          <t>Thresher</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>21.2</v>
+        <v>11.9</v>
       </c>
       <c r="D10" t="n">
-        <v>8.25</v>
+        <v>4.65</v>
       </c>
       <c r="E10" t="n">
-        <v>8.183505965608468</v>
+        <v>3.888647647907649</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>-0.4529595743593035</v>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>0.05585099861600513</v>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
-        <v>-0.7487303292655223</v>
+        <v>-0.679799791432146</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.1640616531249567</v>
-      </c>
-      <c r="R10" t="inlineStr"/>
+        <v>0.277163424977085</v>
+      </c>
+      <c r="R10" t="n">
+        <v>-0.1781765780648783</v>
+      </c>
       <c r="S10" t="n">
-        <v>-0.2657427864752782</v>
-      </c>
-      <c r="T10" t="inlineStr"/>
+        <v>-0.1421253826029762</v>
+      </c>
+      <c r="T10" t="n">
+        <v>-0.347291597132611</v>
+      </c>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="n">
-        <v>9.305525806399229</v>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
-      <c r="X10" t="n">
-        <v>0.3714603208659301</v>
-      </c>
+      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="n">
-        <v>-0.078353664258367</v>
+        <v>9.312726816832022</v>
       </c>
       <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="n">
-        <v>0.9206345506499337</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>0.3729719224889272</v>
-      </c>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1110,7 +1152,7 @@
         <v>12.1</v>
       </c>
       <c r="E11" t="n">
-        <v>11.08924290043289</v>
+        <v>11.34167798941799</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -1124,33 +1166,36 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>0.1579828703094102</v>
+        <v>0.2054413104455245</v>
       </c>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="n">
-        <v>-0.304297599320586</v>
-      </c>
-      <c r="T11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="n">
+        <v>-0.36311150750388</v>
+      </c>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="n">
-        <v>9.643630757640178</v>
-      </c>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
-      <c r="X11" t="n">
-        <v>0.3066636769050058</v>
-      </c>
+      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="n">
-        <v>0.09729163432684355</v>
+        <v>9.615656419295187</v>
       </c>
       <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="n">
-        <v>0.9283680159985847</v>
-      </c>
+      <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="n">
-        <v>0.4051018570465884</v>
+        <v>0.4249210828548864</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.778092981830971</v>
+        <v>0.08352415469680911</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>1.640716281696217</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1.349290470889321</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.349582668870979</v>
       </c>
     </row>
   </sheetData>

</xml_diff>